<commit_message>
Fix formula columns in HTML output (2026-02-17)
</commit_message>
<xml_diff>
--- a/bad_beat_tracker.xlsx
+++ b/bad_beat_tracker.xlsx
@@ -586,11 +586,7 @@
       <c r="B4" s="29" t="n">
         <v>126937.9</v>
       </c>
-      <c r="C4" s="30" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="C4" s="30" t="n"/>
       <c r="D4" s="29" t="n"/>
     </row>
     <row r="5" ht="15" customHeight="1" s="22">
@@ -602,17 +598,14 @@
       <c r="B5" s="29" t="n">
         <v>128353.9</v>
       </c>
-      <c r="C5" s="31">
-        <f>IF(OR(B5="",B4=""),"",B5-B4)</f>
-        <v/>
-      </c>
-      <c r="D5" s="29">
-        <f>IF(OR(B5="",B4=""),"",IF(C5&lt;0,0,IF(B5&lt;150000,C5/0.8,C5/0.6)))</f>
-        <v/>
-      </c>
-      <c r="E5" s="29">
-        <f>IF(D5="","",IF(B5&lt;150000,D5*0.1,D5*0.3))</f>
-        <v/>
+      <c r="C5" s="31" t="n">
+        <v>1416</v>
+      </c>
+      <c r="D5" s="29" t="n">
+        <v>1770</v>
+      </c>
+      <c r="E5" s="29" t="n">
+        <v>177</v>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="22">
@@ -624,17 +617,14 @@
       <c r="B6" s="29" t="n">
         <v>129841.1</v>
       </c>
-      <c r="C6" s="31">
-        <f>IF(OR(B6="",B5=""),"",B6-B5)</f>
-        <v/>
-      </c>
-      <c r="D6" s="29">
-        <f>IF(OR(B6="",B5=""),"",IF(C6&lt;0,0,IF(B6&lt;150000,C6/0.8,C6/0.6)))</f>
-        <v/>
-      </c>
-      <c r="E6" s="29">
-        <f>IF(D6="","",IF(B6&lt;150000,D6*0.1,D6*0.3))</f>
-        <v/>
+      <c r="C6" s="31" t="n">
+        <v>1487.200000000012</v>
+      </c>
+      <c r="D6" s="29" t="n">
+        <v>1859.000000000015</v>
+      </c>
+      <c r="E6" s="29" t="n">
+        <v>185.9000000000015</v>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="22">
@@ -714,9 +704,8 @@
           <t>Total Collected:</t>
         </is>
       </c>
-      <c r="H10" s="35">
-        <f>SUM(D5:D3500)</f>
-        <v/>
+      <c r="H10" s="35" t="n">
+        <v>3629.000000000015</v>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="22">
@@ -756,9 +745,8 @@
           <t>Casino Take:</t>
         </is>
       </c>
-      <c r="H12" s="35">
-        <f>H10*0.1</f>
-        <v/>
+      <c r="H12" s="35" t="n">
+        <v>362.9000000000015</v>
       </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="22">
@@ -835,9 +823,10 @@
           <t>Date:</t>
         </is>
       </c>
-      <c r="H16" s="37">
-        <f>INDEX(A:A,SUMPRODUCT(MAX((D5:D3500=0)*ROW(D5:D3500)))-1)</f>
-        <v/>
+      <c r="H16" s="37" t="inlineStr">
+        <is>
+          <t>2026-02-16</t>
+        </is>
       </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="22">
@@ -860,9 +849,8 @@
           <t>Jackpot:</t>
         </is>
       </c>
-      <c r="H17" s="35">
-        <f>INDEX(B:B,MATCH(H16,A:A,0))</f>
-        <v/>
+      <c r="H17" s="35" t="n">
+        <v>129841.1</v>
       </c>
     </row>
     <row r="18" ht="15" customHeight="1" s="22">
@@ -983,9 +971,8 @@
           <t>Next BBJ:</t>
         </is>
       </c>
-      <c r="H24" s="35">
-        <f>SUMPRODUCT(--(ROW(E5:E200)&gt;MAX(--(D5:D200=0)*ROW(D5:D200))),E5:E200)</f>
-        <v/>
+      <c r="H24" s="35" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="25" ht="15" customHeight="1" s="22">

</xml_diff>

<commit_message>
Update Bad Beat Jackpot data - 2026-02-18
</commit_message>
<xml_diff>
--- a/bad_beat_tracker.xlsx
+++ b/bad_beat_tracker.xlsx
@@ -534,7 +534,7 @@
         </is>
       </c>
       <c r="D1" s="24" t="n">
-        <v>12749.3</v>
+        <v>13541.3</v>
       </c>
       <c r="E1" s="23" t="inlineStr">
         <is>
@@ -543,7 +543,7 @@
       </c>
       <c r="F1" s="25" t="inlineStr">
         <is>
-          <t>2026-02-17</t>
+          <t>2026-02-18</t>
         </is>
       </c>
       <c r="G1" s="26" t="n"/>
@@ -647,19 +647,22 @@
       </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="22">
-      <c r="A8" s="28" t="n"/>
-      <c r="B8" s="29" t="n"/>
-      <c r="C8" s="31">
-        <f>IF(OR(B8="",B7=""),"",B8-B7)</f>
-        <v/>
-      </c>
-      <c r="D8" s="29">
-        <f>IF(OR(B8="",B7=""),"",IF(C8&lt;0,0,IF(B8&lt;150000,C8/0.8,C8/0.6)))</f>
-        <v/>
-      </c>
-      <c r="E8" s="29">
-        <f>IF(D8="","",IF(B8&lt;150000,D8*0.1,D8*0.3))</f>
-        <v/>
+      <c r="A8" s="28" t="inlineStr">
+        <is>
+          <t>2026-02-18</t>
+        </is>
+      </c>
+      <c r="B8" s="29" t="n">
+        <v>13541.3</v>
+      </c>
+      <c r="C8" s="31" t="n">
+        <v>792</v>
+      </c>
+      <c r="D8" s="29" t="n">
+        <v>990</v>
+      </c>
+      <c r="E8" s="29" t="n">
+        <v>99</v>
       </c>
       <c r="G8" s="32" t="inlineStr">
         <is>
@@ -705,7 +708,7 @@
         </is>
       </c>
       <c r="H10" s="35" t="n">
-        <v>3629.000000000015</v>
+        <v>4619.000000000015</v>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="22">
@@ -746,7 +749,7 @@
         </is>
       </c>
       <c r="H12" s="35" t="n">
-        <v>362.9000000000015</v>
+        <v>461.9000000000015</v>
       </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="22">
@@ -972,7 +975,7 @@
         </is>
       </c>
       <c r="H24" s="35" t="n">
-        <v>0</v>
+        <v>99</v>
       </c>
     </row>
     <row r="25" ht="15" customHeight="1" s="22">

</xml_diff>

<commit_message>
Update Bad Beat Jackpot data - 2026-02-19
</commit_message>
<xml_diff>
--- a/bad_beat_tracker.xlsx
+++ b/bad_beat_tracker.xlsx
@@ -534,7 +534,7 @@
         </is>
       </c>
       <c r="D1" s="24" t="n">
-        <v>13541.3</v>
+        <v>14297.3</v>
       </c>
       <c r="E1" s="23" t="inlineStr">
         <is>
@@ -543,7 +543,7 @@
       </c>
       <c r="F1" s="25" t="inlineStr">
         <is>
-          <t>2026-02-18</t>
+          <t>2026-02-19</t>
         </is>
       </c>
       <c r="G1" s="26" t="n"/>
@@ -671,19 +671,22 @@
       </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="22">
-      <c r="A9" s="28" t="n"/>
-      <c r="B9" s="29" t="n"/>
-      <c r="C9" s="31">
-        <f>IF(OR(B9="",B8=""),"",B9-B8)</f>
-        <v/>
-      </c>
-      <c r="D9" s="29">
-        <f>IF(OR(B9="",B8=""),"",IF(C9&lt;0,0,IF(B9&lt;150000,C9/0.8,C9/0.6)))</f>
-        <v/>
-      </c>
-      <c r="E9" s="29">
-        <f>IF(D9="","",IF(B9&lt;150000,D9*0.1,D9*0.3))</f>
-        <v/>
+      <c r="A9" s="28" t="inlineStr">
+        <is>
+          <t>2026-02-19</t>
+        </is>
+      </c>
+      <c r="B9" s="29" t="n">
+        <v>14297.3</v>
+      </c>
+      <c r="C9" s="31" t="n">
+        <v>756</v>
+      </c>
+      <c r="D9" s="29" t="n">
+        <v>945</v>
+      </c>
+      <c r="E9" s="29" t="n">
+        <v>94.5</v>
       </c>
     </row>
     <row r="10" ht="15" customHeight="1" s="22">
@@ -708,7 +711,7 @@
         </is>
       </c>
       <c r="H10" s="35" t="n">
-        <v>4619.000000000015</v>
+        <v>5564.000000000015</v>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="22">
@@ -749,7 +752,7 @@
         </is>
       </c>
       <c r="H12" s="35" t="n">
-        <v>461.9000000000015</v>
+        <v>556.4000000000015</v>
       </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="22">
@@ -975,7 +978,7 @@
         </is>
       </c>
       <c r="H24" s="35" t="n">
-        <v>99</v>
+        <v>193.5</v>
       </c>
     </row>
     <row r="25" ht="15" customHeight="1" s="22">

</xml_diff>

<commit_message>
Update Bad Beat Jackpot data - 2026-02-20
</commit_message>
<xml_diff>
--- a/bad_beat_tracker.xlsx
+++ b/bad_beat_tracker.xlsx
@@ -534,7 +534,7 @@
         </is>
       </c>
       <c r="D1" s="24" t="n">
-        <v>14297.3</v>
+        <v>15007.7</v>
       </c>
       <c r="E1" s="23" t="inlineStr">
         <is>
@@ -543,7 +543,7 @@
       </c>
       <c r="F1" s="25" t="inlineStr">
         <is>
-          <t>2026-02-19</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="G1" s="26" t="n"/>
@@ -690,19 +690,22 @@
       </c>
     </row>
     <row r="10" ht="15" customHeight="1" s="22">
-      <c r="A10" s="28" t="n"/>
-      <c r="B10" s="29" t="n"/>
-      <c r="C10" s="31">
-        <f>IF(OR(B10="",B9=""),"",B10-B9)</f>
-        <v/>
-      </c>
-      <c r="D10" s="29">
-        <f>IF(OR(B10="",B9=""),"",IF(C10&lt;0,0,IF(B10&lt;150000,C10/0.8,C10/0.6)))</f>
-        <v/>
-      </c>
-      <c r="E10" s="29">
-        <f>IF(D10="","",IF(B10&lt;150000,D10*0.1,D10*0.3))</f>
-        <v/>
+      <c r="A10" s="28" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+      <c r="B10" s="29" t="n">
+        <v>15007.7</v>
+      </c>
+      <c r="C10" s="31" t="n">
+        <v>710.4000000000015</v>
+      </c>
+      <c r="D10" s="29" t="n">
+        <v>888.0000000000018</v>
+      </c>
+      <c r="E10" s="29" t="n">
+        <v>88.80000000000018</v>
       </c>
       <c r="F10" s="33" t="n"/>
       <c r="G10" s="34" t="inlineStr">
@@ -711,7 +714,7 @@
         </is>
       </c>
       <c r="H10" s="35" t="n">
-        <v>5564.000000000015</v>
+        <v>6452.000000000016</v>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="22">
@@ -752,7 +755,7 @@
         </is>
       </c>
       <c r="H12" s="35" t="n">
-        <v>556.4000000000015</v>
+        <v>645.2000000000016</v>
       </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="22">
@@ -978,7 +981,7 @@
         </is>
       </c>
       <c r="H24" s="35" t="n">
-        <v>193.5</v>
+        <v>282.3000000000002</v>
       </c>
     </row>
     <row r="25" ht="15" customHeight="1" s="22">

</xml_diff>

<commit_message>
Update Bad Beat Jackpot data - 2026-02-21
</commit_message>
<xml_diff>
--- a/bad_beat_tracker.xlsx
+++ b/bad_beat_tracker.xlsx
@@ -534,7 +534,7 @@
         </is>
       </c>
       <c r="D1" s="24" t="n">
-        <v>15007.7</v>
+        <v>15713.3</v>
       </c>
       <c r="E1" s="23" t="inlineStr">
         <is>
@@ -543,7 +543,7 @@
       </c>
       <c r="F1" s="25" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-02-21</t>
         </is>
       </c>
       <c r="G1" s="26" t="n"/>
@@ -714,23 +714,26 @@
         </is>
       </c>
       <c r="H10" s="35" t="n">
-        <v>6452.000000000016</v>
+        <v>7334.000000000015</v>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="22">
-      <c r="A11" s="28" t="n"/>
-      <c r="B11" s="29" t="n"/>
-      <c r="C11" s="31">
-        <f>IF(OR(B11="",B10=""),"",B11-B10)</f>
-        <v/>
-      </c>
-      <c r="D11" s="29">
-        <f>IF(OR(B11="",B10=""),"",IF(C11&lt;0,0,IF(B11&lt;150000,C11/0.8,C11/0.6)))</f>
-        <v/>
-      </c>
-      <c r="E11" s="29">
-        <f>IF(D11="","",IF(B11&lt;150000,D11*0.1,D11*0.3))</f>
-        <v/>
+      <c r="A11" s="28" t="inlineStr">
+        <is>
+          <t>2026-02-21</t>
+        </is>
+      </c>
+      <c r="B11" s="29" t="n">
+        <v>15713.3</v>
+      </c>
+      <c r="C11" s="31" t="n">
+        <v>705.5999999999985</v>
+      </c>
+      <c r="D11" s="29" t="n">
+        <v>881.9999999999982</v>
+      </c>
+      <c r="E11" s="29" t="n">
+        <v>88.19999999999982</v>
       </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="22">
@@ -755,7 +758,7 @@
         </is>
       </c>
       <c r="H12" s="35" t="n">
-        <v>645.2000000000016</v>
+        <v>733.4000000000015</v>
       </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="22">
@@ -981,7 +984,7 @@
         </is>
       </c>
       <c r="H24" s="35" t="n">
-        <v>282.3000000000002</v>
+        <v>370.5</v>
       </c>
     </row>
     <row r="25" ht="15" customHeight="1" s="22">

</xml_diff>

<commit_message>
Update Bad Beat Jackpot data - 2026-02-22
</commit_message>
<xml_diff>
--- a/bad_beat_tracker.xlsx
+++ b/bad_beat_tracker.xlsx
@@ -534,7 +534,7 @@
         </is>
       </c>
       <c r="D1" s="24" t="n">
-        <v>15713.3</v>
+        <v>16907.7</v>
       </c>
       <c r="E1" s="23" t="inlineStr">
         <is>
@@ -543,7 +543,7 @@
       </c>
       <c r="F1" s="25" t="inlineStr">
         <is>
-          <t>2026-02-21</t>
+          <t>2026-02-22</t>
         </is>
       </c>
       <c r="G1" s="26" t="n"/>
@@ -714,7 +714,7 @@
         </is>
       </c>
       <c r="H10" s="35" t="n">
-        <v>7334.000000000015</v>
+        <v>8827.000000000016</v>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="22">
@@ -737,19 +737,22 @@
       </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="22">
-      <c r="A12" s="28" t="n"/>
-      <c r="B12" s="29" t="n"/>
-      <c r="C12" s="31">
-        <f>IF(OR(B12="",B11=""),"",B12-B11)</f>
-        <v/>
-      </c>
-      <c r="D12" s="29">
-        <f>IF(OR(B12="",B11=""),"",IF(C12&lt;0,0,IF(B12&lt;150000,C12/0.8,C12/0.6)))</f>
-        <v/>
-      </c>
-      <c r="E12" s="29">
-        <f>IF(D12="","",IF(B12&lt;150000,D12*0.1,D12*0.3))</f>
-        <v/>
+      <c r="A12" s="28" t="inlineStr">
+        <is>
+          <t>2026-02-22</t>
+        </is>
+      </c>
+      <c r="B12" s="29" t="n">
+        <v>16907.7</v>
+      </c>
+      <c r="C12" s="31" t="n">
+        <v>1194.400000000001</v>
+      </c>
+      <c r="D12" s="29" t="n">
+        <v>1493.000000000002</v>
+      </c>
+      <c r="E12" s="29" t="n">
+        <v>149.3000000000002</v>
       </c>
       <c r="F12" s="33" t="n"/>
       <c r="G12" s="34" t="inlineStr">
@@ -758,7 +761,7 @@
         </is>
       </c>
       <c r="H12" s="35" t="n">
-        <v>733.4000000000015</v>
+        <v>882.7000000000016</v>
       </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="22">
@@ -984,7 +987,7 @@
         </is>
       </c>
       <c r="H24" s="35" t="n">
-        <v>370.5</v>
+        <v>519.8000000000002</v>
       </c>
     </row>
     <row r="25" ht="15" customHeight="1" s="22">

</xml_diff>

<commit_message>
Update Bad Beat Jackpot data - 2026-02-23
</commit_message>
<xml_diff>
--- a/bad_beat_tracker.xlsx
+++ b/bad_beat_tracker.xlsx
@@ -534,7 +534,7 @@
         </is>
       </c>
       <c r="D1" s="24" t="n">
-        <v>16907.7</v>
+        <v>18190.1</v>
       </c>
       <c r="E1" s="23" t="inlineStr">
         <is>
@@ -543,7 +543,7 @@
       </c>
       <c r="F1" s="25" t="inlineStr">
         <is>
-          <t>2026-02-22</t>
+          <t>2026-02-23</t>
         </is>
       </c>
       <c r="G1" s="26" t="n"/>
@@ -714,7 +714,7 @@
         </is>
       </c>
       <c r="H10" s="35" t="n">
-        <v>8827.000000000016</v>
+        <v>10430.00000000001</v>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="22">
@@ -761,23 +761,26 @@
         </is>
       </c>
       <c r="H12" s="35" t="n">
-        <v>882.7000000000016</v>
+        <v>1043.000000000002</v>
       </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="22">
-      <c r="A13" s="28" t="n"/>
-      <c r="B13" s="29" t="n"/>
-      <c r="C13" s="31">
-        <f>IF(OR(B13="",B12=""),"",B13-B12)</f>
-        <v/>
-      </c>
-      <c r="D13" s="29">
-        <f>IF(OR(B13="",B12=""),"",IF(C13&lt;0,0,IF(B13&lt;150000,C13/0.8,C13/0.6)))</f>
-        <v/>
-      </c>
-      <c r="E13" s="29">
-        <f>IF(D13="","",IF(B13&lt;150000,D13*0.1,D13*0.3))</f>
-        <v/>
+      <c r="A13" s="28" t="inlineStr">
+        <is>
+          <t>2026-02-23</t>
+        </is>
+      </c>
+      <c r="B13" s="29" t="n">
+        <v>18190.1</v>
+      </c>
+      <c r="C13" s="31" t="n">
+        <v>1282.399999999998</v>
+      </c>
+      <c r="D13" s="29" t="n">
+        <v>1602.999999999997</v>
+      </c>
+      <c r="E13" s="29" t="n">
+        <v>160.2999999999997</v>
       </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="22">
@@ -987,7 +990,7 @@
         </is>
       </c>
       <c r="H24" s="35" t="n">
-        <v>519.8000000000002</v>
+        <v>680.0999999999999</v>
       </c>
     </row>
     <row r="25" ht="15" customHeight="1" s="22">

</xml_diff>

<commit_message>
Update Bad Beat Jackpot data - 2026-02-24
</commit_message>
<xml_diff>
--- a/bad_beat_tracker.xlsx
+++ b/bad_beat_tracker.xlsx
@@ -534,7 +534,7 @@
         </is>
       </c>
       <c r="D1" s="24" t="n">
-        <v>18190.1</v>
+        <v>19011.7</v>
       </c>
       <c r="E1" s="23" t="inlineStr">
         <is>
@@ -543,7 +543,7 @@
       </c>
       <c r="F1" s="25" t="inlineStr">
         <is>
-          <t>2026-02-23</t>
+          <t>2026-02-24</t>
         </is>
       </c>
       <c r="G1" s="26" t="n"/>
@@ -714,7 +714,7 @@
         </is>
       </c>
       <c r="H10" s="35" t="n">
-        <v>10430.00000000001</v>
+        <v>11457.00000000002</v>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="22">
@@ -761,7 +761,7 @@
         </is>
       </c>
       <c r="H12" s="35" t="n">
-        <v>1043.000000000002</v>
+        <v>1145.700000000002</v>
       </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="22">
@@ -784,19 +784,22 @@
       </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="22">
-      <c r="A14" s="28" t="n"/>
-      <c r="B14" s="29" t="n"/>
-      <c r="C14" s="31">
-        <f>IF(OR(B14="",B13=""),"",B14-B13)</f>
-        <v/>
-      </c>
-      <c r="D14" s="29">
-        <f>IF(OR(B14="",B13=""),"",IF(C14&lt;0,0,IF(B14&lt;150000,C14/0.8,C14/0.6)))</f>
-        <v/>
-      </c>
-      <c r="E14" s="29">
-        <f>IF(D14="","",IF(B14&lt;150000,D14*0.1,D14*0.3))</f>
-        <v/>
+      <c r="A14" s="28" t="inlineStr">
+        <is>
+          <t>2026-02-24</t>
+        </is>
+      </c>
+      <c r="B14" s="29" t="n">
+        <v>19011.7</v>
+      </c>
+      <c r="C14" s="31" t="n">
+        <v>821.6000000000022</v>
+      </c>
+      <c r="D14" s="29" t="n">
+        <v>1027.000000000003</v>
+      </c>
+      <c r="E14" s="29" t="n">
+        <v>102.7000000000003</v>
       </c>
       <c r="F14" s="33" t="n"/>
       <c r="G14" s="36" t="inlineStr">
@@ -990,7 +993,7 @@
         </is>
       </c>
       <c r="H24" s="35" t="n">
-        <v>680.0999999999999</v>
+        <v>782.8000000000002</v>
       </c>
     </row>
     <row r="25" ht="15" customHeight="1" s="22">

</xml_diff>

<commit_message>
Update Bad Beat Jackpot data - 2026-02-25
</commit_message>
<xml_diff>
--- a/bad_beat_tracker.xlsx
+++ b/bad_beat_tracker.xlsx
@@ -534,7 +534,7 @@
         </is>
       </c>
       <c r="D1" s="24" t="n">
-        <v>19011.7</v>
+        <v>19382.1</v>
       </c>
       <c r="E1" s="23" t="inlineStr">
         <is>
@@ -543,7 +543,7 @@
       </c>
       <c r="F1" s="25" t="inlineStr">
         <is>
-          <t>2026-02-24</t>
+          <t>2026-02-25</t>
         </is>
       </c>
       <c r="G1" s="26" t="n"/>
@@ -714,7 +714,7 @@
         </is>
       </c>
       <c r="H10" s="35" t="n">
-        <v>11457.00000000002</v>
+        <v>11920.00000000001</v>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="22">
@@ -761,7 +761,7 @@
         </is>
       </c>
       <c r="H12" s="35" t="n">
-        <v>1145.700000000002</v>
+        <v>1192.000000000002</v>
       </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="22">
@@ -809,19 +809,22 @@
       </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="22">
-      <c r="A15" s="28" t="n"/>
-      <c r="B15" s="29" t="n"/>
-      <c r="C15" s="31">
-        <f>IF(OR(B15="",B14=""),"",B15-B14)</f>
-        <v/>
-      </c>
-      <c r="D15" s="29">
-        <f>IF(OR(B15="",B14=""),"",IF(C15&lt;0,0,IF(B15&lt;150000,C15/0.8,C15/0.6)))</f>
-        <v/>
-      </c>
-      <c r="E15" s="29">
-        <f>IF(D15="","",IF(B15&lt;150000,D15*0.1,D15*0.3))</f>
-        <v/>
+      <c r="A15" s="28" t="inlineStr">
+        <is>
+          <t>2026-02-25</t>
+        </is>
+      </c>
+      <c r="B15" s="29" t="n">
+        <v>19382.1</v>
+      </c>
+      <c r="C15" s="31" t="n">
+        <v>370.3999999999978</v>
+      </c>
+      <c r="D15" s="29" t="n">
+        <v>462.9999999999973</v>
+      </c>
+      <c r="E15" s="29" t="n">
+        <v>46.29999999999973</v>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1" s="22">
@@ -993,7 +996,7 @@
         </is>
       </c>
       <c r="H24" s="35" t="n">
-        <v>782.8000000000002</v>
+        <v>829.0999999999999</v>
       </c>
     </row>
     <row r="25" ht="15" customHeight="1" s="22">

</xml_diff>